<commit_message>
Atualiza Product Backlog: resolve 5 pendentes do ambiente de teste
Ambiente de Teste & Lançamento passa de 2/14 para 9/14 concluídos:
conta do Administrador do Sistema criada, envio de email (Brevo)
confirmado, armazenamento persistente de imagens configurado (Supabase
Storage/S3), bucket privado de cópias de segurança + agendamento
diário confirmados (cópia feita com sucesso), e ensaio de restauro
validado (22 linhas repostas, 0 divergências). IBAN, NIF/certificado
AGT, domínio próprio e Sentry ficam adiados a pedido explícito; a data
de 2FA obrigatória (14/09/2026) e a série fiscal por fornecedor (só se
aplica quando houver fornecedores reais aprovados) ficam anotadas como
próximos passos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ly7LTXjiZx1TEF6PC9hAd2
</commit_message>
<xml_diff>
--- a/Product_Backlog_KIXIMA.xlsx
+++ b/Product_Backlog_KIXIMA.xlsx
@@ -2683,17 +2683,17 @@
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F60" s="12" t="inlineStr">
         <is>
-          <t>Em curso — a correr assim que a ligação à base ficou estável.</t>
+          <t>Criada via Shell do Render depois de corrigir a DATABASE_URL para o pooler de sessão (porta 5432).</t>
         </is>
       </c>
     </row>
@@ -2713,17 +2713,17 @@
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F61" s="12" t="inlineStr">
         <is>
-          <t>Chave da API já definida; a diagnosticar (provável remetente por verificar).</t>
+          <t>Confirmado: convites e recuperação de senha já chegam aos destinatários.</t>
         </is>
       </c>
     </row>
@@ -2773,17 +2773,17 @@
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
         <is>
-          <t>Sem isto, logótipos e fotos de produto desaparecem a cada deploy.</t>
+          <t>Bucket product-images criado e ligado via STORAGE_PROVIDER=s3 no Render.</t>
         </is>
       </c>
     </row>
@@ -2803,17 +2803,17 @@
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F64" s="12" t="inlineStr">
         <is>
-          <t>STORAGE_BACKUP_BUCKET + BACKUP_CRON.</t>
+          <t>Bucket kixima-backups (privado) criado; "Fazer cópia agora" confirmado com sucesso na Prontidão.</t>
         </is>
       </c>
     </row>
@@ -2833,17 +2833,17 @@
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F65" s="12" t="inlineStr">
         <is>
-          <t>"Uma cópia que nunca foi restaurada não é uma cópia."</t>
+          <t>npm run backup:restore-test — restauro fiel, 22 linhas repostas, 0 divergências.</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
-          <t>Sem isto a plataforma pede transferência sem mostrar para onde.</t>
+          <t>Adiado a pedido do utilizador — dados bancários ainda por definir. Retomar antes do lançamento real.</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="F67" s="12" t="inlineStr">
         <is>
-          <t>A definir antes do lançamento real.</t>
+          <t>Data acordada: 2026-09-14. A confirmar depois de definida no Render.</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
       </c>
       <c r="F68" s="12" t="inlineStr">
         <is>
-          <t>Hoje só configurada para as empresas de demonstração.</t>
+          <t>Tarefa recorrente (não de configuração única): atribuir ao aprovar cada novo fornecedor. Ambiente ainda vazio — sem fornecedores reais aprovados.</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F69" s="12" t="inlineStr">
         <is>
-          <t>Pré-requisito para a faturação sair certificada de facto.</t>
+          <t>Adiado a pedido do utilizador — processo administrativo/regulatório junto da AGT, ainda por iniciar ou confirmar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige percentuais invisíveis no Product Backlog
openpyxl grava toda a fórmula com um valor em cache VAZIO (<v></v>) —
o LibreOffice deste sandbox não consegue recalcular (limitação já
conhecida), e a maioria dos visualizadores que não recalculam fórmulas
mostra essa cache vazia como célula em branco. Era exatamente por isso
que os percentuais (e as contagens) não apareciam.

Corrigido injetando o valor já calculado em Python (a partir da mesma
lista de itens que gera a tabela) diretamente na célula, ao lado da
fórmula — o Excel/LibreOffice continuam a recalcular normalmente se os
dados mudarem, mas agora qualquer visualizador mostra o número certo
de imediato, sem precisar de recalcular primeiro.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ly7LTXjiZx1TEF6PC9hAd2
</commit_message>
<xml_diff>
--- a/Product_Backlog_KIXIMA.xlsx
+++ b/Product_Backlog_KIXIMA.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,12 @@
       <i val="1"/>
       <color rgb="00B8862E"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005B5B5B"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -164,25 +170,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -658,401 +667,406 @@
       </c>
       <c r="C5" s="3">
         <f>COUNTA(Backlog!A2:A71)</f>
-        <v/>
+        <v>70</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Concluído</t>
         </is>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(Backlog!D2:D71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
+        <v>53</v>
+      </c>
+      <c r="D6" s="6">
         <f>C6/$C$5</f>
-        <v/>
+        <v>0.7571428571428571</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Em Curso</t>
         </is>
       </c>
       <c r="C7" s="3">
         <f>COUNTIF(Backlog!D2:D71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
+        <v>2</v>
+      </c>
+      <c r="D7" s="6">
         <f>C7/$C$5</f>
-        <v/>
+        <v>0.02857142857142857</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
       <c r="C8" s="3">
         <f>COUNTIF(Backlog!D2:D71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
+        <v>15</v>
+      </c>
+      <c r="D8" s="6">
         <f>C8/$C$5</f>
-        <v/>
+        <v>0.21428571428571427</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Pendentes por prioridade</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <f>COUNTIFS(Backlog!D2:D71,"Pendente",Backlog!E2:E71,"Alta")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <f>COUNTIFS(Backlog!D2:D71,"Pendente",Backlog!E2:E71,"Média")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <f>COUNTIFS(Backlog!D2:D71,"Pendente",Backlog!E2:E71,"Baixa")</f>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Progresso por Sprint</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Em Curso</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>% Progresso</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B17,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D17" s="9">
+        <v>9</v>
+      </c>
+      <c r="D17" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B17,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E17" s="9">
+        <v>0</v>
+      </c>
+      <c r="E17" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B17,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F17" s="11">
+        <v>0</v>
+      </c>
+      <c r="F17" s="12">
         <f>C17+D17+E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="12">
+        <v>9</v>
+      </c>
+      <c r="G17" s="13">
         <f>C17/F17</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B18,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D18" s="9">
+        <v>5</v>
+      </c>
+      <c r="D18" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B18,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E18" s="9">
+        <v>0</v>
+      </c>
+      <c r="E18" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B18,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F18" s="11">
+        <v>0</v>
+      </c>
+      <c r="F18" s="12">
         <f>C18+D18+E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="12">
+        <v>5</v>
+      </c>
+      <c r="G18" s="13">
         <f>C18/F18</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B19,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D19" s="9">
+        <v>5</v>
+      </c>
+      <c r="D19" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B19,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E19" s="9">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B19,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F19" s="11">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12">
         <f>C19+D19+E19</f>
-        <v/>
-      </c>
-      <c r="G19" s="12">
+        <v>5</v>
+      </c>
+      <c r="G19" s="13">
         <f>C19/F19</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B20,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D20" s="9">
+        <v>3</v>
+      </c>
+      <c r="D20" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B20,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E20" s="9">
+        <v>0</v>
+      </c>
+      <c r="E20" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B20,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F20" s="11">
+        <v>0</v>
+      </c>
+      <c r="F20" s="12">
         <f>C20+D20+E20</f>
-        <v/>
-      </c>
-      <c r="G20" s="12">
+        <v>3</v>
+      </c>
+      <c r="G20" s="13">
         <f>C20/F20</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B21,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D21" s="9">
+        <v>7</v>
+      </c>
+      <c r="D21" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B21,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E21" s="9">
+        <v>0</v>
+      </c>
+      <c r="E21" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B21,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F21" s="11">
+        <v>5</v>
+      </c>
+      <c r="F21" s="12">
         <f>C21+D21+E21</f>
-        <v/>
-      </c>
-      <c r="G21" s="12">
+        <v>12</v>
+      </c>
+      <c r="G21" s="13">
         <f>C21/F21</f>
-        <v/>
+        <v>0.5833333333333334</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B22,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D22" s="9">
+        <v>8</v>
+      </c>
+      <c r="D22" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B22,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E22" s="9">
+        <v>0</v>
+      </c>
+      <c r="E22" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B22,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F22" s="11">
+        <v>5</v>
+      </c>
+      <c r="F22" s="12">
         <f>C22+D22+E22</f>
-        <v/>
-      </c>
-      <c r="G22" s="12">
+        <v>13</v>
+      </c>
+      <c r="G22" s="13">
         <f>C22/F22</f>
-        <v/>
+        <v>0.6153846153846154</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B23,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D23" s="9">
+        <v>5</v>
+      </c>
+      <c r="D23" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B23,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E23" s="9">
+        <v>0</v>
+      </c>
+      <c r="E23" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B23,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F23" s="11">
+        <v>0</v>
+      </c>
+      <c r="F23" s="12">
         <f>C23+D23+E23</f>
-        <v/>
-      </c>
-      <c r="G23" s="12">
+        <v>5</v>
+      </c>
+      <c r="G23" s="13">
         <f>C23/F23</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B24,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D24" s="9">
+        <v>4</v>
+      </c>
+      <c r="D24" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B24,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E24" s="9">
+        <v>0</v>
+      </c>
+      <c r="E24" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B24,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F24" s="11">
+        <v>0</v>
+      </c>
+      <c r="F24" s="12">
         <f>C24+D24+E24</f>
-        <v/>
-      </c>
-      <c r="G24" s="12">
+        <v>4</v>
+      </c>
+      <c r="G24" s="13">
         <f>C24/F24</f>
-        <v/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B25,Backlog!$D$2:$D$71,"Concluído")</f>
-        <v/>
-      </c>
-      <c r="D25" s="9">
+        <v>7</v>
+      </c>
+      <c r="D25" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B25,Backlog!$D$2:$D$71,"Em Curso")</f>
-        <v/>
-      </c>
-      <c r="E25" s="9">
+        <v>2</v>
+      </c>
+      <c r="E25" s="10">
         <f>COUNTIFS(Backlog!$B$2:$B$71,$B25,Backlog!$D$2:$D$71,"Pendente")</f>
-        <v/>
-      </c>
-      <c r="F25" s="11">
+        <v>5</v>
+      </c>
+      <c r="F25" s="12">
         <f>C25+D25+E25</f>
-        <v/>
-      </c>
-      <c r="G25" s="12">
+        <v>14</v>
+      </c>
+      <c r="G25" s="13">
         <f>C25/F25</f>
-        <v/>
+        <v>0.5</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="15">
         <f>SUM(C17:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="14">
+        <v>53</v>
+      </c>
+      <c r="D26" s="15">
         <f>SUM(D17:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="14">
+        <v>2</v>
+      </c>
+      <c r="E26" s="15">
         <f>SUM(E17:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="14">
+        <v>15</v>
+      </c>
+      <c r="F26" s="15">
         <f>SUM(F17:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="15">
+        <v>70</v>
+      </c>
+      <c r="G26" s="16">
         <f>C26/F26</f>
-        <v/>
+        <v>0.7571428571428571</v>
       </c>
     </row>
   </sheetData>
@@ -1087,2132 +1101,2132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Nº</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Item do Backlog</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>Prioridade</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="n">
+      <c r="A2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Catálogo de produtos e serviços (fornecedor publica, comprador explora e compara)</t>
         </is>
       </c>
-      <c r="D2" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E2" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="inlineStr">
         <is>
           <t>Inclui kits, importação em massa via Excel (plano PRO) e API de sincronização de preço/stock.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="n">
+      <c r="A3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>Cotações (RFQ) entre comprador e fornecedor</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>Pedido → resposta com preço/prazo → fecho pelo comprador.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Ciclo completo de Ordens de Compra</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>Aprovação, aceitação, pagamento, execução, entrega, receção e resolução de divergências — 11 estados.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Contratos-quadro e encomendas avulsas (call-offs)</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>Deteção automática no checkout + faturação consolidada periódica (plano PRO).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>Cadastro e aprovação de empresas (due diligence documental)</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>Documentos por tipo de empresa (Cliente/Fornecedora) + apólice obrigatória para fornecedores.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>Gestão de utilizadores, convites e perfis por empresa</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>Perfis: Comprador, Company Admin, Fornecedor, Financeiro.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>Painel do Admin do Sistema (empresas, apólices, contratos, taxas, planos)</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Auditoria (trilho append-only de todas as ações)</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E9" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>Nunca editável/apagável; ator desnormalizado sobrevive à remoção da conta.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>Apólices de seguro (Fornecedor→KIXIMA e KIXIMA→Cliente)</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>Condição de credenciamento para fornecedores.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Autenticação de dois fatores (2FA) — email ou aplicação (TOTP)</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>Obrigatória para Company Admin e Admin do Sistema.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>Bloqueio progressivo de conta por tentativas falhadas de login</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>Por conta, nunca por IP — protege escritórios inteiros atrás do mesmo endereço.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C13" s="19" t="inlineStr">
         <is>
           <t>Admin do Sistema dividido por 6 áreas de permissão + Super Admin</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>Cadastro, Financeiro, Faturação (AGT), Apólices, Suporte, Operação da Plataforma.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>Convite e gestão de Administradores do Sistema (assessores)</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>Nunca cria um Super Admin por convite — exige pelo menos uma área.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>Ecrã de Permissões (bloquear/desbloquear qualquer conta da plataforma)</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="n">
+      <c r="A16" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>Chat de Suporte em tempo real (fila, atribuição, transferência, resolução)</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>Socket.IO autenticado, salas por conversa.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="n">
+      <c r="A17" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
         <is>
           <t>Chat Comercial entre Comprador e Fornecedor</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>Com ou sem contexto (cotação/PO/contrato).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="n">
+      <c r="A18" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>Motor de Trust &amp; Safety (deteção de tentativa de negociar fora da plataforma)</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>6 sinais ponderados; acesso do Suporte a conversa sinalizada é sempre auditado.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="n">
+      <c r="A19" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>Central de Ajuda (FAQ, canais de contacto, estado do sistema)</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>Sistema de Feedback e Avaliações (submissão, moderação, parede pública)</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>Alvo sempre validado contra o histórico real da empresa.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="n">
+      <c r="A21" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="19" t="inlineStr">
         <is>
           <t>Timeline auditável por ordem de compra (histórico completo de eventos)</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>Reaproveita o próprio trilho de auditoria.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="n">
+      <c r="A22" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>Notificações completas de todo o ciclo (criação → conclusão)</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>Antes faltavam avisos em vários passos intermédios.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="n">
+      <c r="A23" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="19" t="inlineStr">
         <is>
           <t>Estado intermédio "Aguardando Pagamento" entre aceite e pagamento</t>
         </is>
       </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E23" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>Estado do enum que existia mas nunca era usado.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>Planos BASE / CORE / PRO com regras por dimensão de empresa (MPME)</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
+      <c r="A25" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="19" t="inlineStr">
         <is>
           <t>Ciclo de vida da subscrição: grace period, avisos escalonados, restrição de funcionalidades</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E25" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Nunca restringe dados/histórico — só funcionalidades premium.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="n">
+      <c r="A26" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="19" t="inlineStr">
         <is>
           <t>Pagamento da subscrição por transferência bancária manual</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E26" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
         <is>
           <t>Todos os planos, incl. PRO — confirmação humana do Admin do Sistema.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n">
+      <c r="A27" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="19" t="inlineStr">
         <is>
           <t>Pagamento automático da subscrição via EMIS/Multicaixa Express</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E27" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
         <is>
           <t>Planos BASE/CORE. Recusa-se a simular sucesso sem credenciais reais.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n">
+      <c r="A28" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C28" s="19" t="inlineStr">
         <is>
           <t>Pagamento automático via PayPay, BAI, BFA, Standard Bank Angola (infraestrutura)</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E28" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
         <is>
           <t>Adaptador genérico honesto — forma provável, por confirmar contra documentação real.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n">
+      <c r="A29" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="19" t="inlineStr">
         <is>
           <t>Conciliação bancária automática (referência única por fatura)</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E29" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" s="18" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr">
         <is>
           <t>Nunca assume pagamento na dúvida — exige referência + valor + moeda exatos.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="n">
+      <c r="A30" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C30" s="19" t="inlineStr">
         <is>
           <t>Taxa de serviço da plataforma (cálculo automático por transação)</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
         <is>
           <t>Fixo até ao limiar, percentual acima.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="n">
+      <c r="A31" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C31" s="19" t="inlineStr">
         <is>
           <t>Credenciais reais EMIS/Multicaixa Express</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="E31" s="20" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F31" s="18" t="inlineStr">
+      <c r="F31" s="19" t="inlineStr">
         <is>
           <t>Depende de contrato comercial com a EMIS.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="n">
+      <c r="A32" s="18" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B32" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C32" s="19" t="inlineStr">
         <is>
           <t>Credenciais reais PayPay</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F32" s="18" t="inlineStr">
+      <c r="F32" s="19" t="inlineStr">
         <is>
           <t>Sem documentação pública da API — depende de acesso direto ao fornecedor.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="n">
+      <c r="A33" s="18" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C33" s="19" t="inlineStr">
         <is>
           <t>Credenciais reais BAI</t>
         </is>
       </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="20" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F33" s="18" t="inlineStr">
+      <c r="F33" s="19" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="n">
+      <c r="A34" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C34" s="19" t="inlineStr">
         <is>
           <t>Credenciais reais BFA</t>
         </is>
       </c>
-      <c r="D34" s="19" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F34" s="19" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="n">
+      <c r="A35" s="18" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="18" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C35" s="18" t="inlineStr">
+      <c r="C35" s="19" t="inlineStr">
         <is>
           <t>Credenciais reais Standard Bank Angola</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E35" s="20" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F35" s="18" t="inlineStr">
+      <c r="F35" s="19" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="n">
+      <c r="A36" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="18" t="inlineStr">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="C36" s="19" t="inlineStr">
         <is>
           <t>Faturação certificada com série e cadeia de integridade por fornecedor</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E36" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
         <is>
           <t>Substituiu uma série global única.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="n">
+      <c r="A37" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="18" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C37" s="18" t="inlineStr">
+      <c r="C37" s="19" t="inlineStr">
         <is>
           <t>Notas de Crédito (documento fiscal com série e cadeia próprias)</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E37" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="18" t="inlineStr">
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
         <is>
           <t>Emitidas só pelo fornecedor; valor nunca excede o saldo por creditar.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="n">
+      <c r="A38" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="18" t="inlineStr">
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="C38" s="19" t="inlineStr">
         <is>
           <t>Linhas de fatura com impostos discriminados (InvoiceLine)</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="18" t="inlineStr">
+      <c r="D38" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
         <is>
           <t>Espelha o modelo oficial impresso da AGT (colunas IEC/IVA/Iselo).</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="n">
+      <c r="A39" s="18" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="18" t="inlineStr">
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C39" s="18" t="inlineStr">
+      <c r="C39" s="19" t="inlineStr">
         <is>
           <t>Recibo como documento fiscal certificado (série e cadeia próprias)</t>
         </is>
       </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="18" t="inlineStr">
+      <c r="D39" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="n">
+      <c r="A40" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="18" t="inlineStr">
+      <c r="B40" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C40" s="18" t="inlineStr">
+      <c r="C40" s="19" t="inlineStr">
         <is>
           <t>Formato do número de documento conforme o exemplo oficial da AGT</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E40" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" s="18" t="inlineStr">
+      <c r="D40" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" s="19" t="inlineStr">
         <is>
           <t>"série.ano/0000001".</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="n">
+      <c r="A41" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="18" t="inlineStr">
+      <c r="B41" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C41" s="18" t="inlineStr">
+      <c r="C41" s="19" t="inlineStr">
         <is>
           <t>Data de adesão à faturação eletrónica por empresa</t>
         </is>
       </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E41" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" s="18" t="inlineStr">
+      <c r="D41" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E41" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="19" t="inlineStr">
         <is>
           <t>Documentos anteriores à data são recusados.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="n">
+      <c r="A42" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="18" t="inlineStr">
+      <c r="B42" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C42" s="18" t="inlineStr">
+      <c r="C42" s="19" t="inlineStr">
         <is>
           <t>Exportação SAF-T com linhas por fatura</t>
         </is>
       </c>
-      <c r="D42" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E42" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F42" s="18" t="inlineStr">
+      <c r="D42" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E42" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
         <is>
           <t>Corrigiu uma lacuna pré-existente (faltavam elementos &lt;Line&gt;).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="n">
+      <c r="A43" s="18" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="18" t="inlineStr">
+      <c r="B43" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C43" s="18" t="inlineStr">
+      <c r="C43" s="19" t="inlineStr">
         <is>
           <t>Verificação de integridade da cadeia de faturação</t>
         </is>
       </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E43" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F43" s="18" t="inlineStr">
+      <c r="D43" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E43" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="19" t="inlineStr">
         <is>
           <t>Deteta buracos na numeração e documentos alterados.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="n">
+      <c r="A44" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="18" t="inlineStr">
+      <c r="B44" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C44" s="19" t="inlineStr">
         <is>
           <t>Ligação real à AGT (assinatura JWS/RS256, submissão em rede)</t>
         </is>
       </c>
-      <c r="D44" s="19" t="inlineStr">
+      <c r="D44" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E44" s="19" t="inlineStr">
+      <c r="E44" s="20" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F44" s="18" t="inlineStr">
+      <c r="F44" s="19" t="inlineStr">
         <is>
           <t>Depende do certificado do programa e credenciais oficiais da AGT.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="n">
+      <c r="A45" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="B45" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>Notas de crédito por linha (hoje só por valor único)</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D45" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E45" s="19" t="inlineStr">
+      <c r="E45" s="20" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F45" s="18" t="inlineStr">
+      <c r="F45" s="19" t="inlineStr">
         <is>
           <t>Decisão de produto em aberto — mudaria o próprio fluxo de crédito.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="n">
+      <c r="A46" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B46" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C46" s="19" t="inlineStr">
         <is>
           <t>Fluxo de anulação de documento fiscal (motivo codificado)</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D46" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E46" s="19" t="inlineStr">
+      <c r="E46" s="20" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F46" s="18" t="inlineStr">
+      <c r="F46" s="19" t="inlineStr">
         <is>
           <t>Não existe nenhum fluxo de anulação hoje.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="n">
+      <c r="A47" s="18" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="18" t="inlineStr">
+      <c r="B47" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>Isenções de IVA reais, taxa reduzida, IEC, Imposto de Selo</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D47" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E47" s="19" t="inlineStr">
+      <c r="E47" s="20" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F47" s="18" t="inlineStr">
+      <c r="F47" s="19" t="inlineStr">
         <is>
           <t>Estrutura de dados pronta; sempre a zero — nenhuma transação real os aciona hoje.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="n">
+      <c r="A48" s="18" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="18" t="inlineStr">
+      <c r="B48" s="19" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
+      <c r="C48" s="19" t="inlineStr">
         <is>
           <t>CAE por linha, multi-estabelecimento, regime de contingência</t>
         </is>
       </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="D48" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E48" s="19" t="inlineStr">
+      <c r="E48" s="20" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F48" s="18" t="inlineStr">
+      <c r="F48" s="19" t="inlineStr">
         <is>
           <t>Fora do âmbito atual — exige ligação real à AGT.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="n">
+      <c r="A49" s="18" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="18" t="inlineStr">
+      <c r="B49" s="19" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="C49" s="19" t="inlineStr">
         <is>
           <t>Homepage corporativa pública com identidade de marca</t>
         </is>
       </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E49" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F49" s="18" t="inlineStr">
+      <c r="D49" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="19" t="inlineStr">
         <is>
           <t>Hero, estatísticas, setores, rede humana, FAQ.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="n">
+      <c r="A50" s="18" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="18" t="inlineStr">
+      <c r="B50" s="19" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
+      <c r="C50" s="19" t="inlineStr">
         <is>
           <t>Estatísticas públicas da plataforma (dados reais, não fictícios)</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E50" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="inlineStr">
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="19" t="inlineStr">
         <is>
           <t>Endpoint público + secção na homepage.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="n">
+      <c r="A51" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="18" t="inlineStr">
+      <c r="B51" s="19" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>Vídeo de demonstração e navegação institucional</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E51" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="inlineStr">
+      <c r="D51" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" s="19" t="inlineStr">
         <is>
           <t>Parcerias, Notícias, Carreiras, Recursos, Termos, Privacidade.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="n">
+      <c r="A52" s="18" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="18" t="inlineStr">
+      <c r="B52" s="19" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
+      <c r="C52" s="19" t="inlineStr">
         <is>
           <t>Internacionalização completa (Português, Inglês, Francês)</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E52" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F52" s="19" t="inlineStr">
         <is>
           <t>0 chaves em falta em EN/FR.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="17" t="n">
+      <c r="A53" s="18" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="18" t="inlineStr">
+      <c r="B53" s="19" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C53" s="18" t="inlineStr">
+      <c r="C53" s="19" t="inlineStr">
         <is>
           <t>Programa Supplier Development (candidatura pública e acompanhamento)</t>
         </is>
       </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E53" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F53" s="18" t="inlineStr">
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="inlineStr">
         <is>
           <t>Aprovação cria a empresa + convite de fundação automaticamente.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="17" t="n">
+      <c r="A54" s="18" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="18" t="inlineStr">
+      <c r="B54" s="19" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C54" s="18" t="inlineStr">
+      <c r="C54" s="19" t="inlineStr">
         <is>
           <t>Manual do Utilizador KIXIMA (.docx)</t>
         </is>
       </c>
-      <c r="D54" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E54" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F54" s="18" t="inlineStr">
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F54" s="19" t="inlineStr">
         <is>
           <t>23 capítulos — todas as personas e transações.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="n">
+      <c r="A55" s="18" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="18" t="inlineStr">
+      <c r="B55" s="19" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C55" s="18" t="inlineStr">
+      <c r="C55" s="19" t="inlineStr">
         <is>
           <t>Guia Visual do Utilizador (.docx, captura de ecrã por página)</t>
         </is>
       </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E55" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F55" s="18" t="inlineStr">
+      <c r="D55" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F55" s="19" t="inlineStr">
         <is>
           <t>75 páginas cobertas, organizadas por perfil.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="17" t="n">
+      <c r="A56" s="18" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="18" t="inlineStr">
+      <c r="B56" s="19" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C56" s="18" t="inlineStr">
+      <c r="C56" s="19" t="inlineStr">
         <is>
           <t>Guia de Ambiente de Teste (AMBIENTE_TESTE.md)</t>
         </is>
       </c>
-      <c r="D56" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E56" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="inlineStr">
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
         <is>
           <t>Infraestrutura isolada para piloto com até 50 utilizadores.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="17" t="n">
+      <c r="A57" s="18" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="18" t="inlineStr">
+      <c r="B57" s="19" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C57" s="18" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
         <is>
           <t>Product Backlog único, por Sprint, com progresso (este ficheiro)</t>
         </is>
       </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E57" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="18" t="inlineStr">
+      <c r="D57" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F57" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="17" t="n">
+      <c r="A58" s="18" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="18" t="inlineStr">
+      <c r="B58" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C58" s="18" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>Infraestrutura do ambiente de teste (Supabase + Render "kixima-teste", isolados da produção)</t>
         </is>
       </c>
-      <c r="D58" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E58" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="18" t="inlineStr">
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F58" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="17" t="n">
+      <c r="A59" s="18" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="18" t="inlineStr">
+      <c r="B59" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C59" s="18" t="inlineStr">
+      <c r="C59" s="19" t="inlineStr">
         <is>
           <t>Ligação estável à base de dados do ambiente de teste</t>
         </is>
       </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E59" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F59" s="18" t="inlineStr">
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F59" s="19" t="inlineStr">
         <is>
           <t>Resolvido: erro de prepared statement do pooler de transação — corrigido usando o pooler de sessão (porta 5432).</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="17" t="n">
+      <c r="A60" s="18" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="18" t="inlineStr">
+      <c r="B60" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C60" s="18" t="inlineStr">
+      <c r="C60" s="19" t="inlineStr">
         <is>
           <t>Criar a conta do Administrador do Sistema no ambiente de teste</t>
         </is>
       </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E60" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="inlineStr">
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F60" s="19" t="inlineStr">
         <is>
           <t>Criada via Shell do Render depois de corrigir a DATABASE_URL para o pooler de sessão (porta 5432).</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="17" t="n">
+      <c r="A61" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="18" t="inlineStr">
+      <c r="B61" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C61" s="18" t="inlineStr">
+      <c r="C61" s="19" t="inlineStr">
         <is>
           <t>Envio de email real a funcionar (Brevo) no ambiente de teste</t>
         </is>
       </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E61" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" s="18" t="inlineStr">
+      <c r="D61" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F61" s="19" t="inlineStr">
         <is>
           <t>Confirmado: convites e recuperação de senha já chegam aos destinatários.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="17" t="n">
+      <c r="A62" s="18" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="18" t="inlineStr">
+      <c r="B62" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C62" s="18" t="inlineStr">
+      <c r="C62" s="19" t="inlineStr">
         <is>
           <t>Armazenamento persistente de imagens (Supabase Storage / S3)</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E62" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" s="18" t="inlineStr">
+      <c r="D62" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F62" s="19" t="inlineStr">
         <is>
           <t>Bucket product-images criado e ligado via STORAGE_PROVIDER=s3 no Render.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="17" t="n">
+      <c r="A63" s="18" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="18" t="inlineStr">
+      <c r="B63" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C63" s="18" t="inlineStr">
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>Bucket privado e cópia de segurança automática agendada</t>
         </is>
       </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E63" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F63" s="18" t="inlineStr">
+      <c r="D63" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F63" s="19" t="inlineStr">
         <is>
           <t>Bucket kixima-backups (privado) criado; "Fazer cópia agora" confirmado com sucesso na Prontidão.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="17" t="n">
+      <c r="A64" s="18" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="18" t="inlineStr">
+      <c r="B64" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C64" s="18" t="inlineStr">
+      <c r="C64" s="19" t="inlineStr">
         <is>
           <t>Ensaio de restauro de uma cópia de segurança</t>
         </is>
       </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E64" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
+      <c r="D64" s="20" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F64" s="19" t="inlineStr">
         <is>
           <t>npm run backup:restore-test — restauro fiel, 22 linhas repostas, 0 divergências.</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="17" t="n">
+      <c r="A65" s="18" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="18" t="inlineStr">
+      <c r="B65" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C65" s="18" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
         <is>
           <t>Piloto com até 50 utilizadores reais</t>
         </is>
       </c>
-      <c r="D65" s="19" t="inlineStr">
+      <c r="D65" s="20" t="inlineStr">
         <is>
           <t>Em Curso</t>
         </is>
       </c>
-      <c r="E65" s="19" t="inlineStr">
+      <c r="E65" s="20" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F65" s="18" t="inlineStr">
+      <c r="F65" s="19" t="inlineStr">
         <is>
           <t>Primeiros utilizadores reais já convidados; falta completar até aos 50.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="17" t="n">
+      <c r="A66" s="18" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="18" t="inlineStr">
+      <c r="B66" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C66" s="18" t="inlineStr">
+      <c r="C66" s="19" t="inlineStr">
         <is>
           <t>Data-limite para 2FA obrigatória (MFA_ENFORCE_FROM)</t>
         </is>
       </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="D66" s="20" t="inlineStr">
         <is>
           <t>Em Curso</t>
         </is>
       </c>
-      <c r="E66" s="19" t="inlineStr">
+      <c r="E66" s="20" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F66" s="18" t="inlineStr">
+      <c r="F66" s="19" t="inlineStr">
         <is>
           <t>Data acordada: 2026-09-14. Falta definir a variável no Render para produzir efeito.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="17" t="n">
+      <c r="A67" s="18" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="18" t="inlineStr">
+      <c r="B67" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C67" s="18" t="inlineStr">
+      <c r="C67" s="19" t="inlineStr">
         <is>
           <t>Conta bancária das subscrições (KIXIMA_BANCO_IBAN)</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D67" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E67" s="19" t="inlineStr">
+      <c r="E67" s="20" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F67" s="18" t="inlineStr">
+      <c r="F67" s="19" t="inlineStr">
         <is>
           <t>Adiado a pedido do utilizador — dados bancários ainda por definir. Retomar antes do lançamento real.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="17" t="n">
+      <c r="A68" s="18" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="18" t="inlineStr">
+      <c r="B68" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C68" s="18" t="inlineStr">
+      <c r="C68" s="19" t="inlineStr">
         <is>
           <t>NIF da KIXIMA e certificado do programa junto da AGT</t>
         </is>
       </c>
-      <c r="D68" s="19" t="inlineStr">
+      <c r="D68" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E68" s="19" t="inlineStr">
+      <c r="E68" s="20" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F68" s="18" t="inlineStr">
+      <c r="F68" s="19" t="inlineStr">
         <is>
           <t>Adiado a pedido do utilizador — processo administrativo/regulatório junto da AGT, ainda por iniciar ou confirmar.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="17" t="n">
+      <c r="A69" s="18" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="18" t="inlineStr">
+      <c r="B69" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C69" s="18" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>Série de faturação certificada por cada fornecedor real</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
+      <c r="D69" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E69" s="19" t="inlineStr">
+      <c r="E69" s="20" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F69" s="18" t="inlineStr">
+      <c r="F69" s="19" t="inlineStr">
         <is>
           <t>Tarefa recorrente (não de configuração única): atribuir ao aprovar cada novo fornecedor. Ambiente ainda vazio — sem fornecedores reais aprovados.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="17" t="n">
+      <c r="A70" s="18" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="18" t="inlineStr">
+      <c r="B70" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C70" s="18" t="inlineStr">
+      <c r="C70" s="19" t="inlineStr">
         <is>
           <t>Domínio próprio (ex.: app.kixima.co.ao)</t>
         </is>
       </c>
-      <c r="D70" s="19" t="inlineStr">
+      <c r="D70" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E70" s="19" t="inlineStr">
+      <c r="E70" s="20" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F70" s="18" t="inlineStr">
+      <c r="F70" s="19" t="inlineStr">
         <is>
           <t>Opcional — atualizar APP_URL depois de ligado.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="17" t="n">
+      <c r="A71" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="18" t="inlineStr">
+      <c r="B71" s="19" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C71" s="18" t="inlineStr">
+      <c r="C71" s="19" t="inlineStr">
         <is>
           <t>Rastreio de erros em produção (Sentry)</t>
         </is>
       </c>
-      <c r="D71" s="19" t="inlineStr">
+      <c r="D71" s="20" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E71" s="19" t="inlineStr">
+      <c r="E71" s="20" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F71" s="18" t="inlineStr">
+      <c r="F71" s="19" t="inlineStr">
         <is>
           <t>Opcional, recomendado antes de abrir a operadoras.</t>
         </is>

</xml_diff>

<commit_message>
Backlog: aplica a mesma identidade visual da folha Resumo aos itens
A folha Backlog passa a mostrar os 70 itens agrupados visualmente por
Sprint (cabeçalho a azul-marinho por secção, com uma barra de
estatísticas logo a seguir: progresso do Sprint e contagem/percentual
de Concluído/Em Curso/Pendente), mais uma legenda geral no topo com o
mesmo resumo para o backlog inteiro. Cada linha de item continua colorida
automaticamente por Estado (verde/âmbar/vermelho) e por Prioridade.
As secções de cada Sprint ficam agrupáveis (outline) para recolher os
itens e ver só os cabeçalhos. Continua um único ficheiro (Resumo +
Backlog), sem nenhuma aba ou ficheiro novo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ly7LTXjiZx1TEF6PC9hAd2
</commit_message>
<xml_diff>
--- a/Product_Backlog_KIXIMA.xlsx
+++ b/Product_Backlog_KIXIMA.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,48 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005B5B5B"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -104,14 +146,8 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001B2A4A"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -121,6 +157,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001B2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F1EA"/>
       </patternFill>
     </fill>
     <fill>
@@ -170,39 +211,60 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="21" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -327,21 +389,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Backlog" displayName="Backlog" ref="A1:F71" headerRowCount="1">
-  <autoFilter ref="A1:F71"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Nº"/>
-    <tableColumn id="2" name="Sprint"/>
-    <tableColumn id="3" name="Item do Backlog"/>
-    <tableColumn id="4" name="Estado"/>
-    <tableColumn id="5" name="Prioridade"/>
-    <tableColumn id="6" name="Notas"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -666,7 +713,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>COUNTA(Backlog!A2:A71)</f>
+        <f>C6+C7+C8</f>
         <v>70</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -682,7 +729,7 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <f>COUNTIF(Backlog!D2:D71,"Concluído")</f>
+        <f>COUNTIF(Backlog!D2:D101,"Concluído")</f>
         <v>53</v>
       </c>
       <c r="D6" s="6">
@@ -697,7 +744,7 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <f>COUNTIF(Backlog!D2:D71,"Em Curso")</f>
+        <f>COUNTIF(Backlog!D2:D101,"Em Curso")</f>
         <v>2</v>
       </c>
       <c r="D7" s="6">
@@ -712,7 +759,7 @@
         </is>
       </c>
       <c r="C8" s="3">
-        <f>COUNTIF(Backlog!D2:D71,"Pendente")</f>
+        <f>COUNTIF(Backlog!D2:D101,"Pendente")</f>
         <v>15</v>
       </c>
       <c r="D8" s="6">
@@ -734,7 +781,7 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIFS(Backlog!D2:D71,"Pendente",Backlog!E2:E71,"Alta")</f>
+        <f>COUNTIFS(Backlog!D2:D101,"Pendente",Backlog!E2:E101,"Alta")</f>
         <v>4</v>
       </c>
     </row>
@@ -745,7 +792,7 @@
         </is>
       </c>
       <c r="C12" s="10">
-        <f>COUNTIFS(Backlog!D2:D71,"Pendente",Backlog!E2:E71,"Média")</f>
+        <f>COUNTIFS(Backlog!D2:D101,"Pendente",Backlog!E2:E101,"Média")</f>
         <v>5</v>
       </c>
     </row>
@@ -756,7 +803,7 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIFS(Backlog!D2:D71,"Pendente",Backlog!E2:E71,"Baixa")</f>
+        <f>COUNTIFS(Backlog!D2:D101,"Pendente",Backlog!E2:E101,"Baixa")</f>
         <v>6</v>
       </c>
     </row>
@@ -806,15 +853,15 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B17,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B17,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>9</v>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B17,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B17,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B17,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B17,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>0</v>
       </c>
       <c r="F17" s="12">
@@ -833,15 +880,15 @@
         </is>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B18,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B18,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>5</v>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B18,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B18,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E18" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B18,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B18,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>0</v>
       </c>
       <c r="F18" s="12">
@@ -860,15 +907,15 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B19,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B19,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>5</v>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B19,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B19,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B19,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B19,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>0</v>
       </c>
       <c r="F19" s="12">
@@ -887,15 +934,15 @@
         </is>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B20,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B20,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>3</v>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B20,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B20,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E20" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B20,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B20,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>0</v>
       </c>
       <c r="F20" s="12">
@@ -914,15 +961,15 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B21,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B21,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>7</v>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B21,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B21,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B21,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B21,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>5</v>
       </c>
       <c r="F21" s="12">
@@ -941,15 +988,15 @@
         </is>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B22,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B22,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>8</v>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B22,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B22,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E22" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B22,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B22,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>5</v>
       </c>
       <c r="F22" s="12">
@@ -968,15 +1015,15 @@
         </is>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B23,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B23,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>5</v>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B23,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B23,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E23" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B23,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B23,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>0</v>
       </c>
       <c r="F23" s="12">
@@ -995,15 +1042,15 @@
         </is>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B24,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B24,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>4</v>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B24,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B24,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>0</v>
       </c>
       <c r="E24" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B24,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B24,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>0</v>
       </c>
       <c r="F24" s="12">
@@ -1022,15 +1069,15 @@
         </is>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B25,Backlog!$D$2:$D$71,"Concluído")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B25,Backlog!$D$2:$D$101,"Concluído")</f>
         <v>7</v>
       </c>
       <c r="D25" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B25,Backlog!$D$2:$D$71,"Em Curso")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B25,Backlog!$D$2:$D$101,"Em Curso")</f>
         <v>2</v>
       </c>
       <c r="E25" s="10">
-        <f>COUNTIFS(Backlog!$B$2:$B$71,$B25,Backlog!$D$2:$D$71,"Pendente")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$101,$B25,Backlog!$D$2:$D$101,"Pendente")</f>
         <v>5</v>
       </c>
       <c r="F25" s="12">
@@ -1086,14 +1133,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col hidden="1" width="30" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -1133,2107 +1180,2454 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="n">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>RESUMO GERAL DO BACKLOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 53 (76%)</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 2 (3%)</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 15 (21%)</t>
+        </is>
+      </c>
+      <c r="E3" s="22" t="inlineStr">
+        <is>
+          <t>Total: 70 itens</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 1 — Núcleo do Marketplace</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Progresso: 100%</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 9 (100%)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>9 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" outlineLevel="1">
+      <c r="A7" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Catálogo de produtos e serviços (fornecedor publica, comprador explora e compara)</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E2" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F2" s="19" t="inlineStr">
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>Inclui kits, importação em massa via Excel (plano PRO) e API de sincronização de preço/stock.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="18" t="n">
+    <row r="8" outlineLevel="1">
+      <c r="A8" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>Cotações (RFQ) entre comprador e fornecedor</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F3" s="19" t="inlineStr">
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
         <is>
           <t>Pedido → resposta com preço/prazo → fecho pelo comprador.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="18" t="n">
+    <row r="9" outlineLevel="1">
+      <c r="A9" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Ciclo completo de Ordens de Compra</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>Aprovação, aceitação, pagamento, execução, entrega, receção e resolução de divergências — 11 estados.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="18" t="n">
+    <row r="10" outlineLevel="1">
+      <c r="A10" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>Contratos-quadro e encomendas avulsas (call-offs)</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E5" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
         <is>
           <t>Deteção automática no checkout + faturação consolidada periódica (plano PRO).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="18" t="n">
+    <row r="11" outlineLevel="1">
+      <c r="A11" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>Cadastro e aprovação de empresas (due diligence documental)</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
         <is>
           <t>Documentos por tipo de empresa (Cliente/Fornecedora) + apólice obrigatória para fornecedores.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="18" t="n">
+    <row r="12" outlineLevel="1">
+      <c r="A12" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>Gestão de utilizadores, convites e perfis por empresa</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="inlineStr">
         <is>
           <t>Perfis: Comprador, Company Admin, Fornecedor, Financeiro.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="18" t="n">
+    <row r="13" outlineLevel="1">
+      <c r="A13" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Painel do Admin do Sistema (empresas, apólices, contratos, taxas, planos)</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="n">
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" outlineLevel="1">
+      <c r="A14" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>Auditoria (trilho append-only de todas as ações)</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
         <is>
           <t>Nunca editável/apagável; ator desnormalizado sobrevive à remoção da conta.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="18" t="n">
+    <row r="15" outlineLevel="1">
+      <c r="A15" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Sprint 1 — Núcleo do Marketplace</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Apólices de seguro (Fornecedor→KIXIMA e KIXIMA→Cliente)</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>Condição de credenciamento para fornecedores.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="18" t="n">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 2 — Segurança &amp; Controlo de Acesso</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Progresso: 100%</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 5 (100%)</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>5 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" outlineLevel="1">
+      <c r="A19" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>Autenticação de dois fatores (2FA) — email ou aplicação (TOTP)</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="19" t="inlineStr">
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
         <is>
           <t>Obrigatória para Company Admin e Admin do Sistema.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="18" t="n">
+    <row r="20" outlineLevel="1">
+      <c r="A20" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>Bloqueio progressivo de conta por tentativas falhadas de login</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="inlineStr">
         <is>
           <t>Por conta, nunca por IP — protege escritórios inteiros atrás do mesmo endereço.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="18" t="n">
+    <row r="21" outlineLevel="1">
+      <c r="A21" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>Admin do Sistema dividido por 6 áreas de permissão + Super Admin</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="19" t="inlineStr">
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="inlineStr">
         <is>
           <t>Cadastro, Financeiro, Faturação (AGT), Apólices, Suporte, Operação da Plataforma.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="18" t="n">
+    <row r="22" outlineLevel="1">
+      <c r="A22" s="25" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>Convite e gestão de Administradores do Sistema (assessores)</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="inlineStr">
         <is>
           <t>Nunca cria um Super Admin por convite — exige pelo menos uma área.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="18" t="n">
+    <row r="23" outlineLevel="1">
+      <c r="A23" s="25" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Sprint 2 — Segurança &amp; Controlo de Acesso</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>Ecrã de Permissões (bloquear/desbloquear qualquer conta da plataforma)</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 3 — Suporte &amp; Confiança</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Progresso: 100%</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 5 (100%)</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>5 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" outlineLevel="1">
+      <c r="A27" s="25" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C27" s="27" t="inlineStr">
         <is>
           <t>Chat de Suporte em tempo real (fila, atribuição, transferência, resolução)</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="inlineStr">
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="inlineStr">
         <is>
           <t>Socket.IO autenticado, salas por conversa.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="18" t="n">
+    <row r="28" outlineLevel="1">
+      <c r="A28" s="25" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B28" s="26" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C28" s="27" t="inlineStr">
         <is>
           <t>Chat Comercial entre Comprador e Fornecedor</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="inlineStr">
         <is>
           <t>Com ou sem contexto (cotação/PO/contrato).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="n">
+    <row r="29" outlineLevel="1">
+      <c r="A29" s="25" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C29" s="27" t="inlineStr">
         <is>
           <t>Motor de Trust &amp; Safety (deteção de tentativa de negociar fora da plataforma)</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="inlineStr">
         <is>
           <t>6 sinais ponderados; acesso do Suporte a conversa sinalizada é sempre auditado.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="18" t="n">
+    <row r="30" outlineLevel="1">
+      <c r="A30" s="25" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C30" s="27" t="inlineStr">
         <is>
           <t>Central de Ajuda (FAQ, canais de contacto, estado do sistema)</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="n">
+      <c r="D30" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" outlineLevel="1">
+      <c r="A31" s="25" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Sprint 3 — Suporte &amp; Confiança</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C31" s="27" t="inlineStr">
         <is>
           <t>Sistema de Feedback e Avaliações (submissão, moderação, parede pública)</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E20" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
+      <c r="D31" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="inlineStr">
         <is>
           <t>Alvo sempre validado contra o histórico real da empresa.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="18" t="n">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 4 — Ordens de Compra</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Progresso: 100%</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 3 (100%)</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>3 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" outlineLevel="1">
+      <c r="A35" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Timeline auditável por ordem de compra (histórico completo de eventos)</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="inlineStr">
         <is>
           <t>Reaproveita o próprio trilho de auditoria.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="18" t="n">
+    <row r="36" outlineLevel="1">
+      <c r="A36" s="25" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>Notificações completas de todo o ciclo (criação → conclusão)</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr">
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="inlineStr">
         <is>
           <t>Antes faltavam avisos em vários passos intermédios.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="18" t="n">
+    <row r="37" outlineLevel="1">
+      <c r="A37" s="25" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>Sprint 4 — Ordens de Compra</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C37" s="27" t="inlineStr">
         <is>
           <t>Estado intermédio "Aguardando Pagamento" entre aceite e pagamento</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E23" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="inlineStr">
+      <c r="D37" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="inlineStr">
         <is>
           <t>Estado do enum que existia mas nunca era usado.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="18" t="n">
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 5 — Subscrições &amp; Pagamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Progresso: 58%</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 7 (58%)</t>
+        </is>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 5 (42%)</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>12 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" outlineLevel="1">
+      <c r="A41" s="25" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C41" s="27" t="inlineStr">
         <is>
           <t>Planos BASE / CORE / PRO com regras por dimensão de empresa (MPME)</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E24" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="18" t="n">
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" outlineLevel="1">
+      <c r="A42" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="19" t="inlineStr">
+      <c r="B42" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C42" s="27" t="inlineStr">
         <is>
           <t>Ciclo de vida da subscrição: grace period, avisos escalonados, restrição de funcionalidades</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E25" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="inlineStr">
         <is>
           <t>Nunca restringe dados/histórico — só funcionalidades premium.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="18" t="n">
+    <row r="43" outlineLevel="1">
+      <c r="A43" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C43" s="27" t="inlineStr">
         <is>
           <t>Pagamento da subscrição por transferência bancária manual</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E43" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="inlineStr">
         <is>
           <t>Todos os planos, incl. PRO — confirmação humana do Admin do Sistema.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="18" t="n">
+    <row r="44" outlineLevel="1">
+      <c r="A44" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="19" t="inlineStr">
+      <c r="B44" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C44" s="27" t="inlineStr">
         <is>
           <t>Pagamento automático da subscrição via EMIS/Multicaixa Express</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E27" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="19" t="inlineStr">
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="inlineStr">
         <is>
           <t>Planos BASE/CORE. Recusa-se a simular sucesso sem credenciais reais.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="18" t="n">
+    <row r="45" outlineLevel="1">
+      <c r="A45" s="25" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="19" t="inlineStr">
+      <c r="B45" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr">
+      <c r="C45" s="27" t="inlineStr">
         <is>
           <t>Pagamento automático via PayPay, BAI, BFA, Standard Bank Angola (infraestrutura)</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E28" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E45" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="inlineStr">
         <is>
           <t>Adaptador genérico honesto — forma provável, por confirmar contra documentação real.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="18" t="n">
+    <row r="46" outlineLevel="1">
+      <c r="A46" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="19" t="inlineStr">
+      <c r="B46" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="C46" s="27" t="inlineStr">
         <is>
           <t>Conciliação bancária automática (referência única por fatura)</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E29" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" s="19" t="inlineStr">
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E46" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="inlineStr">
         <is>
           <t>Nunca assume pagamento na dúvida — exige referência + valor + moeda exatos.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="18" t="n">
+    <row r="47" outlineLevel="1">
+      <c r="A47" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B47" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C30" s="19" t="inlineStr">
+      <c r="C47" s="27" t="inlineStr">
         <is>
           <t>Taxa de serviço da plataforma (cálculo automático por transação)</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E30" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" s="19" t="inlineStr">
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E47" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F47" s="27" t="inlineStr">
         <is>
           <t>Fixo até ao limiar, percentual acima.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="18" t="n">
+    <row r="48" outlineLevel="1">
+      <c r="A48" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="19" t="inlineStr">
+      <c r="B48" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C48" s="27" t="inlineStr">
         <is>
           <t>Credenciais reais EMIS/Multicaixa Express</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D48" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="E48" s="26" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F31" s="19" t="inlineStr">
+      <c r="F48" s="27" t="inlineStr">
         <is>
           <t>Depende de contrato comercial com a EMIS.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="18" t="n">
+    <row r="49" outlineLevel="1">
+      <c r="A49" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="19" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
+      <c r="C49" s="27" t="inlineStr">
         <is>
           <t>Credenciais reais PayPay</t>
         </is>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D49" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F32" s="19" t="inlineStr">
+      <c r="F49" s="27" t="inlineStr">
         <is>
           <t>Sem documentação pública da API — depende de acesso direto ao fornecedor.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="n">
+    <row r="50" outlineLevel="1">
+      <c r="A50" s="25" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B50" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C50" s="27" t="inlineStr">
         <is>
           <t>Credenciais reais BAI</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D50" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E33" s="20" t="inlineStr">
+      <c r="E50" s="26" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F33" s="19" t="inlineStr">
+      <c r="F50" s="27" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="18" t="n">
+    <row r="51" outlineLevel="1">
+      <c r="A51" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="19" t="inlineStr">
+      <c r="B51" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C34" s="19" t="inlineStr">
+      <c r="C51" s="27" t="inlineStr">
         <is>
           <t>Credenciais reais BFA</t>
         </is>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D51" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="E51" s="26" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F34" s="19" t="inlineStr">
+      <c r="F51" s="27" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="18" t="n">
+    <row r="52" outlineLevel="1">
+      <c r="A52" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="19" t="inlineStr">
+      <c r="B52" s="26" t="inlineStr">
         <is>
           <t>Sprint 5 — Subscrições &amp; Pagamentos</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C52" s="27" t="inlineStr">
         <is>
           <t>Credenciais reais Standard Bank Angola</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D52" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E52" s="26" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F35" s="19" t="inlineStr">
+      <c r="F52" s="27" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="18" t="n">
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>Progresso: 62%</t>
+        </is>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 8 (62%)</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 5 (38%)</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="inlineStr">
+        <is>
+          <t>13 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" outlineLevel="1">
+      <c r="A56" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B56" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="C56" s="27" t="inlineStr">
         <is>
           <t>Faturação certificada com série e cadeia de integridade por fornecedor</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E36" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="19" t="inlineStr">
+      <c r="D56" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E56" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="inlineStr">
         <is>
           <t>Substituiu uma série global única.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="18" t="n">
+    <row r="57" outlineLevel="1">
+      <c r="A57" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="19" t="inlineStr">
+      <c r="B57" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="C57" s="27" t="inlineStr">
         <is>
           <t>Notas de Crédito (documento fiscal com série e cadeia próprias)</t>
         </is>
       </c>
-      <c r="D37" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E37" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F37" s="19" t="inlineStr">
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E57" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F57" s="27" t="inlineStr">
         <is>
           <t>Emitidas só pelo fornecedor; valor nunca excede o saldo por creditar.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="18" t="n">
+    <row r="58" outlineLevel="1">
+      <c r="A58" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="19" t="inlineStr">
+      <c r="B58" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="C58" s="27" t="inlineStr">
         <is>
           <t>Linhas de fatura com impostos discriminados (InvoiceLine)</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E38" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" s="19" t="inlineStr">
+      <c r="D58" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F58" s="27" t="inlineStr">
         <is>
           <t>Espelha o modelo oficial impresso da AGT (colunas IEC/IVA/Iselo).</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="18" t="n">
+    <row r="59" outlineLevel="1">
+      <c r="A59" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="19" t="inlineStr">
+      <c r="B59" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C39" s="19" t="inlineStr">
+      <c r="C59" s="27" t="inlineStr">
         <is>
           <t>Recibo como documento fiscal certificado (série e cadeia próprias)</t>
         </is>
       </c>
-      <c r="D39" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E39" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="18" t="n">
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E59" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" outlineLevel="1">
+      <c r="A60" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="19" t="inlineStr">
+      <c r="B60" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
+      <c r="C60" s="27" t="inlineStr">
         <is>
           <t>Formato do número de documento conforme o exemplo oficial da AGT</t>
         </is>
       </c>
-      <c r="D40" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E40" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" s="19" t="inlineStr">
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E60" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F60" s="27" t="inlineStr">
         <is>
           <t>"série.ano/0000001".</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="18" t="n">
+    <row r="61" outlineLevel="1">
+      <c r="A61" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B61" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
+      <c r="C61" s="27" t="inlineStr">
         <is>
           <t>Data de adesão à faturação eletrónica por empresa</t>
         </is>
       </c>
-      <c r="D41" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E41" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" s="19" t="inlineStr">
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E61" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F61" s="27" t="inlineStr">
         <is>
           <t>Documentos anteriores à data são recusados.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="18" t="n">
+    <row r="62" outlineLevel="1">
+      <c r="A62" s="25" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="19" t="inlineStr">
+      <c r="B62" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C42" s="19" t="inlineStr">
+      <c r="C62" s="27" t="inlineStr">
         <is>
           <t>Exportação SAF-T com linhas por fatura</t>
         </is>
       </c>
-      <c r="D42" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E42" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F42" s="19" t="inlineStr">
+      <c r="D62" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E62" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F62" s="27" t="inlineStr">
         <is>
           <t>Corrigiu uma lacuna pré-existente (faltavam elementos &lt;Line&gt;).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="18" t="n">
+    <row r="63" outlineLevel="1">
+      <c r="A63" s="25" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="19" t="inlineStr">
+      <c r="B63" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C63" s="27" t="inlineStr">
         <is>
           <t>Verificação de integridade da cadeia de faturação</t>
         </is>
       </c>
-      <c r="D43" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E43" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F43" s="19" t="inlineStr">
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E63" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="inlineStr">
         <is>
           <t>Deteta buracos na numeração e documentos alterados.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="18" t="n">
+    <row r="64" outlineLevel="1">
+      <c r="A64" s="25" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="19" t="inlineStr">
+      <c r="B64" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C44" s="19" t="inlineStr">
+      <c r="C64" s="27" t="inlineStr">
         <is>
           <t>Ligação real à AGT (assinatura JWS/RS256, submissão em rede)</t>
         </is>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D64" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E44" s="20" t="inlineStr">
+      <c r="E64" s="26" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F44" s="19" t="inlineStr">
+      <c r="F64" s="27" t="inlineStr">
         <is>
           <t>Depende do certificado do programa e credenciais oficiais da AGT.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="18" t="n">
+    <row r="65" outlineLevel="1">
+      <c r="A65" s="25" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="19" t="inlineStr">
+      <c r="B65" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C65" s="27" t="inlineStr">
         <is>
           <t>Notas de crédito por linha (hoje só por valor único)</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D65" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E65" s="26" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F45" s="19" t="inlineStr">
+      <c r="F65" s="27" t="inlineStr">
         <is>
           <t>Decisão de produto em aberto — mudaria o próprio fluxo de crédito.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="18" t="n">
+    <row r="66" outlineLevel="1">
+      <c r="A66" s="25" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="19" t="inlineStr">
+      <c r="B66" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr">
+      <c r="C66" s="27" t="inlineStr">
         <is>
           <t>Fluxo de anulação de documento fiscal (motivo codificado)</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D66" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="E66" s="26" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F46" s="19" t="inlineStr">
+      <c r="F66" s="27" t="inlineStr">
         <is>
           <t>Não existe nenhum fluxo de anulação hoje.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="18" t="n">
+    <row r="67" outlineLevel="1">
+      <c r="A67" s="25" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="19" t="inlineStr">
+      <c r="B67" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C67" s="27" t="inlineStr">
         <is>
           <t>Isenções de IVA reais, taxa reduzida, IEC, Imposto de Selo</t>
         </is>
       </c>
-      <c r="D47" s="20" t="inlineStr">
+      <c r="D67" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E47" s="20" t="inlineStr">
+      <c r="E67" s="26" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F47" s="19" t="inlineStr">
+      <c r="F67" s="27" t="inlineStr">
         <is>
           <t>Estrutura de dados pronta; sempre a zero — nenhuma transação real os aciona hoje.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="18" t="n">
+    <row r="68" outlineLevel="1">
+      <c r="A68" s="25" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="19" t="inlineStr">
+      <c r="B68" s="26" t="inlineStr">
         <is>
           <t>Sprint 6 — Faturação &amp; Fiscalidade (AGT)</t>
         </is>
       </c>
-      <c r="C48" s="19" t="inlineStr">
+      <c r="C68" s="27" t="inlineStr">
         <is>
           <t>CAE por linha, multi-estabelecimento, regime de contingência</t>
         </is>
       </c>
-      <c r="D48" s="20" t="inlineStr">
+      <c r="D68" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E48" s="20" t="inlineStr">
+      <c r="E68" s="26" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F48" s="19" t="inlineStr">
+      <c r="F68" s="27" t="inlineStr">
         <is>
           <t>Fora do âmbito atual — exige ligação real à AGT.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="18" t="n">
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 7 — Página Institucional &amp; Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="19" t="inlineStr">
+        <is>
+          <t>Progresso: 100%</t>
+        </is>
+      </c>
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 5 (100%)</t>
+        </is>
+      </c>
+      <c r="C71" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D71" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>5 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" outlineLevel="1">
+      <c r="A72" s="25" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="19" t="inlineStr">
+      <c r="B72" s="26" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C49" s="19" t="inlineStr">
+      <c r="C72" s="27" t="inlineStr">
         <is>
           <t>Homepage corporativa pública com identidade de marca</t>
         </is>
       </c>
-      <c r="D49" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F49" s="19" t="inlineStr">
+      <c r="D72" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E72" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="27" t="inlineStr">
         <is>
           <t>Hero, estatísticas, setores, rede humana, FAQ.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="18" t="n">
+    <row r="73" outlineLevel="1">
+      <c r="A73" s="25" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="19" t="inlineStr">
+      <c r="B73" s="26" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C50" s="19" t="inlineStr">
+      <c r="C73" s="27" t="inlineStr">
         <is>
           <t>Estatísticas públicas da plataforma (dados reais, não fictícios)</t>
         </is>
       </c>
-      <c r="D50" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E50" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F50" s="19" t="inlineStr">
+      <c r="D73" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E73" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="27" t="inlineStr">
         <is>
           <t>Endpoint público + secção na homepage.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="18" t="n">
+    <row r="74" outlineLevel="1">
+      <c r="A74" s="25" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="19" t="inlineStr">
+      <c r="B74" s="26" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C74" s="27" t="inlineStr">
         <is>
           <t>Vídeo de demonstração e navegação institucional</t>
         </is>
       </c>
-      <c r="D51" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E51" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F51" s="19" t="inlineStr">
+      <c r="D74" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E74" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="27" t="inlineStr">
         <is>
           <t>Parcerias, Notícias, Carreiras, Recursos, Termos, Privacidade.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="18" t="n">
+    <row r="75" outlineLevel="1">
+      <c r="A75" s="25" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="19" t="inlineStr">
+      <c r="B75" s="26" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C52" s="19" t="inlineStr">
+      <c r="C75" s="27" t="inlineStr">
         <is>
           <t>Internacionalização completa (Português, Inglês, Francês)</t>
         </is>
       </c>
-      <c r="D52" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E52" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="19" t="inlineStr">
+      <c r="D75" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E75" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F75" s="27" t="inlineStr">
         <is>
           <t>0 chaves em falta em EN/FR.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="18" t="n">
+    <row r="76" outlineLevel="1">
+      <c r="A76" s="25" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="19" t="inlineStr">
+      <c r="B76" s="26" t="inlineStr">
         <is>
           <t>Sprint 7 — Página Institucional &amp; Marketing</t>
         </is>
       </c>
-      <c r="C53" s="19" t="inlineStr">
+      <c r="C76" s="27" t="inlineStr">
         <is>
           <t>Programa Supplier Development (candidatura pública e acompanhamento)</t>
         </is>
       </c>
-      <c r="D53" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E53" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F53" s="19" t="inlineStr">
+      <c r="D76" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E76" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F76" s="27" t="inlineStr">
         <is>
           <t>Aprovação cria a empresa + convite de fundação automaticamente.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="18" t="n">
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 8 — Documentação</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="19" t="inlineStr">
+        <is>
+          <t>Progresso: 100%</t>
+        </is>
+      </c>
+      <c r="B79" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 4 (100%)</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="D79" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 0 (0%)</t>
+        </is>
+      </c>
+      <c r="E79" s="24" t="inlineStr">
+        <is>
+          <t>4 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" outlineLevel="1">
+      <c r="A80" s="25" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="19" t="inlineStr">
+      <c r="B80" s="26" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C54" s="19" t="inlineStr">
+      <c r="C80" s="27" t="inlineStr">
         <is>
           <t>Manual do Utilizador KIXIMA (.docx)</t>
         </is>
       </c>
-      <c r="D54" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E54" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F54" s="19" t="inlineStr">
+      <c r="D80" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E80" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="27" t="inlineStr">
         <is>
           <t>23 capítulos — todas as personas e transações.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="18" t="n">
+    <row r="81" outlineLevel="1">
+      <c r="A81" s="25" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="19" t="inlineStr">
+      <c r="B81" s="26" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C55" s="19" t="inlineStr">
+      <c r="C81" s="27" t="inlineStr">
         <is>
           <t>Guia Visual do Utilizador (.docx, captura de ecrã por página)</t>
         </is>
       </c>
-      <c r="D55" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E55" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F55" s="19" t="inlineStr">
+      <c r="D81" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E81" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="27" t="inlineStr">
         <is>
           <t>75 páginas cobertas, organizadas por perfil.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="18" t="n">
+    <row r="82" outlineLevel="1">
+      <c r="A82" s="25" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="19" t="inlineStr">
+      <c r="B82" s="26" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C56" s="19" t="inlineStr">
+      <c r="C82" s="27" t="inlineStr">
         <is>
           <t>Guia de Ambiente de Teste (AMBIENTE_TESTE.md)</t>
         </is>
       </c>
-      <c r="D56" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E56" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F56" s="19" t="inlineStr">
+      <c r="D82" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E82" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="27" t="inlineStr">
         <is>
           <t>Infraestrutura isolada para piloto com até 50 utilizadores.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="18" t="n">
+    <row r="83" outlineLevel="1">
+      <c r="A83" s="25" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="19" t="inlineStr">
+      <c r="B83" s="26" t="inlineStr">
         <is>
           <t>Sprint 8 — Documentação</t>
         </is>
       </c>
-      <c r="C57" s="19" t="inlineStr">
+      <c r="C83" s="27" t="inlineStr">
         <is>
           <t>Product Backlog único, por Sprint, com progresso (este ficheiro)</t>
         </is>
       </c>
-      <c r="D57" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="18" t="n">
+      <c r="D83" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E83" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F83" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="20" t="inlineStr">
+        <is>
+          <t>Progresso: 50%</t>
+        </is>
+      </c>
+      <c r="B86" s="19" t="inlineStr">
+        <is>
+          <t>Concluído: 7 (50%)</t>
+        </is>
+      </c>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>Em Curso: 2 (14%)</t>
+        </is>
+      </c>
+      <c r="D86" s="21" t="inlineStr">
+        <is>
+          <t>Pendente: 5 (36%)</t>
+        </is>
+      </c>
+      <c r="E86" s="24" t="inlineStr">
+        <is>
+          <t>14 itens neste Sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" outlineLevel="1">
+      <c r="A87" s="25" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="19" t="inlineStr">
+      <c r="B87" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C58" s="19" t="inlineStr">
+      <c r="C87" s="27" t="inlineStr">
         <is>
           <t>Infraestrutura do ambiente de teste (Supabase + Render "kixima-teste", isolados da produção)</t>
         </is>
       </c>
-      <c r="D58" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E58" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="18" t="n">
+      <c r="D87" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E87" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" outlineLevel="1">
+      <c r="A88" s="25" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="19" t="inlineStr">
+      <c r="B88" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C59" s="19" t="inlineStr">
+      <c r="C88" s="27" t="inlineStr">
         <is>
           <t>Ligação estável à base de dados do ambiente de teste</t>
         </is>
       </c>
-      <c r="D59" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F59" s="19" t="inlineStr">
+      <c r="D88" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E88" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="inlineStr">
         <is>
           <t>Resolvido: erro de prepared statement do pooler de transação — corrigido usando o pooler de sessão (porta 5432).</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="18" t="n">
+    <row r="89" outlineLevel="1">
+      <c r="A89" s="25" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="19" t="inlineStr">
+      <c r="B89" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C60" s="19" t="inlineStr">
+      <c r="C89" s="27" t="inlineStr">
         <is>
           <t>Criar a conta do Administrador do Sistema no ambiente de teste</t>
         </is>
       </c>
-      <c r="D60" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E60" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F60" s="19" t="inlineStr">
+      <c r="D89" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E89" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="inlineStr">
         <is>
           <t>Criada via Shell do Render depois de corrigir a DATABASE_URL para o pooler de sessão (porta 5432).</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="18" t="n">
+    <row r="90" outlineLevel="1">
+      <c r="A90" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="19" t="inlineStr">
+      <c r="B90" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C61" s="19" t="inlineStr">
+      <c r="C90" s="27" t="inlineStr">
         <is>
           <t>Envio de email real a funcionar (Brevo) no ambiente de teste</t>
         </is>
       </c>
-      <c r="D61" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" s="19" t="inlineStr">
+      <c r="D90" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E90" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="inlineStr">
         <is>
           <t>Confirmado: convites e recuperação de senha já chegam aos destinatários.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="18" t="n">
+    <row r="91" outlineLevel="1">
+      <c r="A91" s="25" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="19" t="inlineStr">
+      <c r="B91" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C62" s="19" t="inlineStr">
+      <c r="C91" s="27" t="inlineStr">
         <is>
           <t>Armazenamento persistente de imagens (Supabase Storage / S3)</t>
         </is>
       </c>
-      <c r="D62" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E62" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" s="19" t="inlineStr">
+      <c r="D91" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E91" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F91" s="27" t="inlineStr">
         <is>
           <t>Bucket product-images criado e ligado via STORAGE_PROVIDER=s3 no Render.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="18" t="n">
+    <row r="92" outlineLevel="1">
+      <c r="A92" s="25" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="19" t="inlineStr">
+      <c r="B92" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C63" s="19" t="inlineStr">
+      <c r="C92" s="27" t="inlineStr">
         <is>
           <t>Bucket privado e cópia de segurança automática agendada</t>
         </is>
       </c>
-      <c r="D63" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F63" s="19" t="inlineStr">
+      <c r="D92" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E92" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F92" s="27" t="inlineStr">
         <is>
           <t>Bucket kixima-backups (privado) criado; "Fazer cópia agora" confirmado com sucesso na Prontidão.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="18" t="n">
+    <row r="93" outlineLevel="1">
+      <c r="A93" s="25" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="19" t="inlineStr">
+      <c r="B93" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C64" s="19" t="inlineStr">
+      <c r="C93" s="27" t="inlineStr">
         <is>
           <t>Ensaio de restauro de uma cópia de segurança</t>
         </is>
       </c>
-      <c r="D64" s="20" t="inlineStr">
-        <is>
-          <t>Concluído</t>
-        </is>
-      </c>
-      <c r="E64" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F64" s="19" t="inlineStr">
+      <c r="D93" s="26" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="E93" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F93" s="27" t="inlineStr">
         <is>
           <t>npm run backup:restore-test — restauro fiel, 22 linhas repostas, 0 divergências.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="18" t="n">
+    <row r="94" outlineLevel="1">
+      <c r="A94" s="25" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="19" t="inlineStr">
+      <c r="B94" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C65" s="19" t="inlineStr">
+      <c r="C94" s="27" t="inlineStr">
         <is>
           <t>Piloto com até 50 utilizadores reais</t>
         </is>
       </c>
-      <c r="D65" s="20" t="inlineStr">
+      <c r="D94" s="26" t="inlineStr">
         <is>
           <t>Em Curso</t>
         </is>
       </c>
-      <c r="E65" s="20" t="inlineStr">
+      <c r="E94" s="26" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F65" s="19" t="inlineStr">
+      <c r="F94" s="27" t="inlineStr">
         <is>
           <t>Primeiros utilizadores reais já convidados; falta completar até aos 50.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="18" t="n">
+    <row r="95" outlineLevel="1">
+      <c r="A95" s="25" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="19" t="inlineStr">
+      <c r="B95" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C66" s="19" t="inlineStr">
+      <c r="C95" s="27" t="inlineStr">
         <is>
           <t>Data-limite para 2FA obrigatória (MFA_ENFORCE_FROM)</t>
         </is>
       </c>
-      <c r="D66" s="20" t="inlineStr">
+      <c r="D95" s="26" t="inlineStr">
         <is>
           <t>Em Curso</t>
         </is>
       </c>
-      <c r="E66" s="20" t="inlineStr">
+      <c r="E95" s="26" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F66" s="19" t="inlineStr">
+      <c r="F95" s="27" t="inlineStr">
         <is>
           <t>Data acordada: 2026-09-14. Falta definir a variável no Render para produzir efeito.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="18" t="n">
+    <row r="96" outlineLevel="1">
+      <c r="A96" s="25" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="19" t="inlineStr">
+      <c r="B96" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="C96" s="27" t="inlineStr">
         <is>
           <t>Conta bancária das subscrições (KIXIMA_BANCO_IBAN)</t>
         </is>
       </c>
-      <c r="D67" s="20" t="inlineStr">
+      <c r="D96" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E67" s="20" t="inlineStr">
+      <c r="E96" s="26" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F67" s="19" t="inlineStr">
+      <c r="F96" s="27" t="inlineStr">
         <is>
           <t>Adiado a pedido do utilizador — dados bancários ainda por definir. Retomar antes do lançamento real.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="18" t="n">
+    <row r="97" outlineLevel="1">
+      <c r="A97" s="25" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="19" t="inlineStr">
+      <c r="B97" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C68" s="19" t="inlineStr">
+      <c r="C97" s="27" t="inlineStr">
         <is>
           <t>NIF da KIXIMA e certificado do programa junto da AGT</t>
         </is>
       </c>
-      <c r="D68" s="20" t="inlineStr">
+      <c r="D97" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E68" s="20" t="inlineStr">
+      <c r="E97" s="26" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F68" s="19" t="inlineStr">
+      <c r="F97" s="27" t="inlineStr">
         <is>
           <t>Adiado a pedido do utilizador — processo administrativo/regulatório junto da AGT, ainda por iniciar ou confirmar.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="18" t="n">
+    <row r="98" outlineLevel="1">
+      <c r="A98" s="25" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="19" t="inlineStr">
+      <c r="B98" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C69" s="19" t="inlineStr">
+      <c r="C98" s="27" t="inlineStr">
         <is>
           <t>Série de faturação certificada por cada fornecedor real</t>
         </is>
       </c>
-      <c r="D69" s="20" t="inlineStr">
+      <c r="D98" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E69" s="20" t="inlineStr">
+      <c r="E98" s="26" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="F69" s="19" t="inlineStr">
+      <c r="F98" s="27" t="inlineStr">
         <is>
           <t>Tarefa recorrente (não de configuração única): atribuir ao aprovar cada novo fornecedor. Ambiente ainda vazio — sem fornecedores reais aprovados.</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="18" t="n">
+    <row r="99" outlineLevel="1">
+      <c r="A99" s="25" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="19" t="inlineStr">
+      <c r="B99" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C70" s="19" t="inlineStr">
+      <c r="C99" s="27" t="inlineStr">
         <is>
           <t>Domínio próprio (ex.: app.kixima.co.ao)</t>
         </is>
       </c>
-      <c r="D70" s="20" t="inlineStr">
+      <c r="D99" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E70" s="20" t="inlineStr">
+      <c r="E99" s="26" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F70" s="19" t="inlineStr">
+      <c r="F99" s="27" t="inlineStr">
         <is>
           <t>Opcional — atualizar APP_URL depois de ligado.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="18" t="n">
+    <row r="100" outlineLevel="1">
+      <c r="A100" s="25" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="19" t="inlineStr">
+      <c r="B100" s="26" t="inlineStr">
         <is>
           <t>Sprint 9 — Ambiente de Teste &amp; Lançamento</t>
         </is>
       </c>
-      <c r="C71" s="19" t="inlineStr">
+      <c r="C100" s="27" t="inlineStr">
         <is>
           <t>Rastreio de erros em produção (Sentry)</t>
         </is>
       </c>
-      <c r="D71" s="20" t="inlineStr">
+      <c r="D100" s="26" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="E71" s="20" t="inlineStr">
+      <c r="E100" s="26" t="inlineStr">
         <is>
           <t>Baixa</t>
         </is>
       </c>
-      <c r="F71" s="19" t="inlineStr">
+      <c r="F100" s="27" t="inlineStr">
         <is>
           <t>Opcional, recomendado antes de abrir a operadoras.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D71">
+  <mergeCells count="10">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A85:F85"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D1:D101">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Concluído"</formula>
     </cfRule>
@@ -3244,7 +3638,7 @@
       <formula>"Pendente"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E71">
+  <conditionalFormatting sqref="E1:E101">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
       <formula>"Alta"</formula>
     </cfRule>
@@ -3253,8 +3647,5 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>